<commit_message>
Pace Report: eliminar ADR del gráfico
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/auditoria_dashboard.xlsx
+++ b/output/auditoria_dashboard.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-05-25 18:43</t>
+          <t>2026-05-26 09:22</t>
         </is>
       </c>
     </row>
@@ -20424,10 +20424,10 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>650.04</v>
+        <v>1211.4</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>650.04</v>
+        <v>1211.4</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Dashboard v4: consola ejecutiva premium
- 4 KPI cards grandes (Revenue/Occupancy/ADR Pace + Airbnb Health)
- Pace Report hero con ADR dots sobre barras (offset fijo, sin eje Y)
- Resumen automático sobre el Pace Report
- Evolución: 2 columnas (anual: ingresos/ocu/ADR barras+líneas | mensual: mismo)
- Huecos simplificados a tarjetas compactas informativas
- Airbnb Health: rating + superhost + cancelaciones + conversión
- Lead Time colapsado en Analytics avanzados
- Ingresos mensuales: línea → barras
- drawOcuAnnual y drawADRAnnual nuevos

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/auditoria_dashboard.xlsx
+++ b/output/auditoria_dashboard.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-05-26 09:22</t>
+          <t>2026-05-26 10:31</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Ningún cambio respecto al baseline del 2026-05-25.</t>
+          <t>Ningún cambio respecto al baseline del 2026-05-26.</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr"/>
@@ -11545,7 +11545,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Ningún cambio respecto al baseline del 2026-05-25.</t>
+          <t>Ningún cambio respecto al baseline del 2026-05-26.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr"/>

</xml_diff>